<commit_message>
add 4 new report
</commit_message>
<xml_diff>
--- a/Traveloka_DataAutomation_Portal_Expedia/Data/ListReport.xlsx
+++ b/Traveloka_DataAutomation_Portal_Expedia/Data/ListReport.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Kalyana\dataautomation_personal\Traveloka_DataAutomation_Portal_Expedia\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DF96517-4FDB-4DAC-84FA-56EA3D55ACBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18DA004E-C47B-44B4-A17E-B40E0ABE903E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3852" yWindow="3852" windowWidth="21588" windowHeight="10620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23232" windowHeight="11496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="24">
   <si>
     <t>BPID</t>
   </si>
@@ -86,6 +86,18 @@
   </si>
   <si>
     <t>HT0254</t>
+  </si>
+  <si>
+    <t>HT0405</t>
+  </si>
+  <si>
+    <t>HT0406</t>
+  </si>
+  <si>
+    <t>HT0407</t>
+  </si>
+  <si>
+    <t>HT0408</t>
   </si>
 </sst>
 </file>
@@ -127,13 +139,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -414,17 +430,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.5" customWidth="1"/>
+    <col min="1" max="1" width="11.44140625" customWidth="1"/>
     <col min="2" max="2" width="49" style="1" customWidth="1"/>
-    <col min="3" max="3" width="7" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.25" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.88671875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -441,7 +457,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
@@ -458,7 +474,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -475,7 +491,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -489,6 +505,74 @@
         <v>2</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="5">
+        <v>613254</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="5">
+        <v>613255</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="5">
+        <v>613256</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="5">
+        <v>613257</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -504,14 +588,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{876B688B-8D39-4F48-905C-6944AEF29D9D}">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="34.75" style="1" customWidth="1"/>
-    <col min="3" max="5" width="11.25" style="1" customWidth="1"/>
+    <col min="2" max="2" width="34.77734375" style="1" customWidth="1"/>
+    <col min="3" max="5" width="11.21875" style="1" customWidth="1"/>
     <col min="6" max="6" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -534,7 +618,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
@@ -553,7 +637,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -576,7 +660,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>

</xml_diff>